<commit_message>
just login is remaining
</commit_message>
<xml_diff>
--- a/banking_app/bank_records.xlsx
+++ b/banking_app/bank_records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7b434e343d34443a/Desktop/Python_ Training/banking_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2B597847148DEEC3A877D0B34B1510344D078D22" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5657D35D-3117-4362-8D19-0D0705374CBE}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_56BD2AE4930F45450D6BBBD94A7B902F7C7584AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5D40305-EC5C-446F-85D3-7D494A1F06D7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Account No</t>
   </si>
@@ -47,6 +47,39 @@
   </si>
   <si>
     <t>Date-Time</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">harshad </t>
+  </si>
+  <si>
+    <t>0606</t>
+  </si>
+  <si>
+    <t>ad43fef7</t>
+  </si>
+  <si>
+    <t>Opening</t>
+  </si>
+  <si>
+    <t>2026-09-08 10:28:08</t>
+  </si>
+  <si>
+    <t>12346</t>
+  </si>
+  <si>
+    <t>rohini</t>
+  </si>
+  <si>
+    <t>1460</t>
+  </si>
+  <si>
+    <t>4009aaa7</t>
+  </si>
+  <si>
+    <t>2026-09-08 10:29:03</t>
   </si>
 </sst>
 </file>
@@ -386,8 +419,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.21875" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="9" max="9" width="17.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -416,6 +457,64 @@
       </c>
       <c r="I1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2">
+        <v>50000</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>50000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3">
+        <v>10000</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>10000</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>